<commit_message>
format templates and update web UI
</commit_message>
<xml_diff>
--- a/data/Baseline_cover_TEMPLATE.xlsx
+++ b/data/Baseline_cover_TEMPLATE.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp.sharepoint.com/sites/usgs-carbonate_budget_restoration_tool/Shared Documents/Carbonate Budget Tool Collaboration/Carbonate_Budget_Tool_Code/CarbonateBudgetRestorationTool/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\__git\CBuRT\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="161" documentId="8_{04AD622C-265A-44CF-BFA2-BE05B0EF88AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D156C810-3A22-4106-9F1F-189A3F56C56C}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE8193C0-727E-4A27-AB34-04D4A18EB61B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="1" xr2:uid="{0278FB9D-D97A-43A8-AA68-A0B70EFAF30B}"/>
+    <workbookView xWindow="57480" yWindow="22020" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{0278FB9D-D97A-43A8-AA68-A0B70EFAF30B}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="3" r:id="rId1"/>
@@ -910,13 +910,17 @@
   <dimension ref="A1:K1"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="3" width="13.73046875" customWidth="1"/>
-    <col min="4" max="4" width="14.19921875" customWidth="1"/>
-    <col min="5" max="5" width="13.59765625" customWidth="1"/>
-    <col min="6" max="6" width="10.265625" customWidth="1"/>
-    <col min="7" max="7" width="9.46484375" customWidth="1"/>
-    <col min="8" max="8" width="10.265625" customWidth="1"/>
-    <col min="9" max="9" width="14.06640625" customWidth="1"/>
+    <col min="1" max="1" width="5.796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.46484375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.1328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.86328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.1328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.53125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.3984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.86328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.06640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.45">
@@ -1401,6 +1405,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="797e7fd4-719a-42b3-b312-968ffa9058ad">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="811eef35-9bdd-441e-81aa-50455f68c6c3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000AA90A7536739341825FB392424435FB" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ca57789ecb406bb7a99068f68ac4c0ed">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="797e7fd4-719a-42b3-b312-968ffa9058ad" xmlns:ns3="811eef35-9bdd-441e-81aa-50455f68c6c3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="89dc4794f4784a0bac47690674a3da53" ns2:_="" ns3:_="">
     <xsd:import namespace="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
@@ -1595,17 +1610,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="797e7fd4-719a-42b3-b312-968ffa9058ad">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="811eef35-9bdd-441e-81aa-50455f68c6c3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D6BB395-747F-41BC-A23A-168993E4FE92}">
   <ds:schemaRefs>
@@ -1615,6 +1619,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9D3406C-31AD-4E38-96F6-B0246BC4EAE6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
+    <ds:schemaRef ds:uri="811eef35-9bdd-441e-81aa-50455f68c6c3"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D5B4E66-2F53-40AB-B6DF-59838CE46951}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1633,17 +1648,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9D3406C-31AD-4E38-96F6-B0246BC4EAE6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
-    <ds:schemaRef ds:uri="811eef35-9bdd-441e-81aa-50455f68c6c3"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{6dd02d64-b7f3-43f7-a145-cfd68d338edf}" enabled="1" method="Standard" siteId="{0693b5ba-4b18-4d7b-9341-f32f400a5494}" removed="0"/>

</xml_diff>

<commit_message>
add example data and update map interface
</commit_message>
<xml_diff>
--- a/data/Baseline_cover_TEMPLATE.xlsx
+++ b/data/Baseline_cover_TEMPLATE.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\__git\CBuRT\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE8193C0-727E-4A27-AB34-04D4A18EB61B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8D7FFE5-3CA2-48E9-8B47-7A7148B2308C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="22020" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{0278FB9D-D97A-43A8-AA68-A0B70EFAF30B}"/>
+    <workbookView xWindow="2175" yWindow="2175" windowWidth="21600" windowHeight="11332" activeTab="1" xr2:uid="{0278FB9D-D97A-43A8-AA68-A0B70EFAF30B}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="3" r:id="rId1"/>
     <sheet name="Coral Cover input" sheetId="1" r:id="rId2"/>
-    <sheet name="Taxon list" sheetId="2" r:id="rId3"/>
+    <sheet name="Taxa" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -974,7 +974,7 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{101649E4-CD8D-4DAA-89FC-8D6C93B48E30}">
           <x14:formula1>
-            <xm:f>'Taxon list'!$A$2:$A$80</xm:f>
+            <xm:f>Taxa!$A$2:$A$80</xm:f>
           </x14:formula1>
           <xm:sqref>A2:A1048576</xm:sqref>
         </x14:dataValidation>
@@ -1396,26 +1396,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="797e7fd4-719a-42b3-b312-968ffa9058ad">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="811eef35-9bdd-441e-81aa-50455f68c6c3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000AA90A7536739341825FB392424435FB" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ca57789ecb406bb7a99068f68ac4c0ed">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="797e7fd4-719a-42b3-b312-968ffa9058ad" xmlns:ns3="811eef35-9bdd-441e-81aa-50455f68c6c3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="89dc4794f4784a0bac47690674a3da53" ns2:_="" ns3:_="">
     <xsd:import namespace="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
@@ -1610,26 +1590,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D6BB395-747F-41BC-A23A-168993E4FE92}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="797e7fd4-719a-42b3-b312-968ffa9058ad">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="811eef35-9bdd-441e-81aa-50455f68c6c3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9D3406C-31AD-4E38-96F6-B0246BC4EAE6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
-    <ds:schemaRef ds:uri="811eef35-9bdd-441e-81aa-50455f68c6c3"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D5B4E66-2F53-40AB-B6DF-59838CE46951}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1648,6 +1629,25 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9D3406C-31AD-4E38-96F6-B0246BC4EAE6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
+    <ds:schemaRef ds:uri="811eef35-9bdd-441e-81aa-50455f68c6c3"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D6BB395-747F-41BC-A23A-168993E4FE92}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{6dd02d64-b7f3-43f7-a145-cfd68d338edf}" enabled="1" method="Standard" siteId="{0693b5ba-4b18-4d7b-9341-f32f400a5494}" removed="0"/>

</xml_diff>

<commit_message>
improve .xlsx template input filters
</commit_message>
<xml_diff>
--- a/data/Baseline_cover_TEMPLATE.xlsx
+++ b/data/Baseline_cover_TEMPLATE.xlsx
@@ -8,15 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\__git\CBuRT\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8D7FFE5-3CA2-48E9-8B47-7A7148B2308C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{336DB45F-BBF4-41AC-B528-ECD6973AF431}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2175" yWindow="2175" windowWidth="21600" windowHeight="11332" activeTab="1" xr2:uid="{0278FB9D-D97A-43A8-AA68-A0B70EFAF30B}"/>
+    <workbookView xWindow="4478" yWindow="1905" windowWidth="21600" windowHeight="11340" activeTab="1" xr2:uid="{0278FB9D-D97A-43A8-AA68-A0B70EFAF30B}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="3" r:id="rId1"/>
     <sheet name="Coral Cover input" sheetId="1" r:id="rId2"/>
     <sheet name="Taxa" sheetId="2" r:id="rId3"/>
+    <sheet name="Metadata" sheetId="4" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="RangeA">Metadata!$B$2:$B$4</definedName>
+    <definedName name="RangeDRTO">Metadata!$B$5:$B$7</definedName>
+    <definedName name="SEFCRI">Metadata!$B$8</definedName>
+    <definedName name="SubregionList">Metadata!$A$2:$A$5</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -41,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="117">
   <si>
     <t>Acropora cervicornis</t>
   </si>
@@ -400,6 +407,48 @@
   </si>
   <si>
     <t>•  Please provide a point of contact (POC) first and last name and email for the baseline site data so that we can contact you with questions, if necessary</t>
+  </si>
+  <si>
+    <t>Habitat_FK</t>
+  </si>
+  <si>
+    <t>DryTortugas</t>
+  </si>
+  <si>
+    <t>Inshore</t>
+  </si>
+  <si>
+    <t>LowerKeys</t>
+  </si>
+  <si>
+    <t>MidChannel</t>
+  </si>
+  <si>
+    <t>MiddleKeys</t>
+  </si>
+  <si>
+    <t>Offshore</t>
+  </si>
+  <si>
+    <t>UpperKeys</t>
+  </si>
+  <si>
+    <t>Bank</t>
+  </si>
+  <si>
+    <t>Biscayne</t>
+  </si>
+  <si>
+    <t>Lagoon</t>
+  </si>
+  <si>
+    <t>SoutheastFlorida</t>
+  </si>
+  <si>
+    <t>ForeReef</t>
+  </si>
+  <si>
+    <t>SEFCRI</t>
   </si>
 </sst>
 </file>
@@ -962,7 +1011,7 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D1048576" xr:uid="{268EBEEC-525C-485A-BCB7-2F826408B174}">
-      <formula1>"Inshore, MidChannel, Offshore, Bank, Lagoon, ForeReef"</formula1>
+      <formula1>IF(C2="DryTortugas",        RangeDRTO,    IF(ISNUMBER(MATCH(C2, SubregionList, 0)),        RangeA,     SEFCRI))</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C1048576" xr:uid="{2551E9F4-EAD3-4C0C-A0CF-00F9C4CBBDD7}">
       <formula1>"DryTortugas, LowerKeys,MiddleKeys, UpperKeys, Biscayne, SoutheastFlorida"</formula1>
@@ -1395,7 +1444,98 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58E31873-3B71-4C96-9888-7DA8F3D3EA70}">
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>110</v>
+      </c>
+      <c r="B4" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>112</v>
+      </c>
+      <c r="B5" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>114</v>
+      </c>
+      <c r="B6" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>104</v>
+      </c>
+      <c r="B7" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="B8" t="s">
+        <v>116</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="797e7fd4-719a-42b3-b312-968ffa9058ad">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="811eef35-9bdd-441e-81aa-50455f68c6c3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000AA90A7536739341825FB392424435FB" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ca57789ecb406bb7a99068f68ac4c0ed">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="797e7fd4-719a-42b3-b312-968ffa9058ad" xmlns:ns3="811eef35-9bdd-441e-81aa-50455f68c6c3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="89dc4794f4784a0bac47690674a3da53" ns2:_="" ns3:_="">
     <xsd:import namespace="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
@@ -1590,27 +1730,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="797e7fd4-719a-42b3-b312-968ffa9058ad">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="811eef35-9bdd-441e-81aa-50455f68c6c3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D6BB395-747F-41BC-A23A-168993E4FE92}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9D3406C-31AD-4E38-96F6-B0246BC4EAE6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
+    <ds:schemaRef ds:uri="811eef35-9bdd-441e-81aa-50455f68c6c3"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D5B4E66-2F53-40AB-B6DF-59838CE46951}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1629,25 +1768,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9D3406C-31AD-4E38-96F6-B0246BC4EAE6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
-    <ds:schemaRef ds:uri="811eef35-9bdd-441e-81aa-50455f68c6c3"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D6BB395-747F-41BC-A23A-168993E4FE92}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{6dd02d64-b7f3-43f7-a145-cfd68d338edf}" enabled="1" method="Standard" siteId="{0693b5ba-4b18-4d7b-9341-f32f400a5494}" removed="0"/>

</xml_diff>